<commit_message>
feat: actualiza simulador fiscal con excel final, parametrización de comisiones, combobox premium y validación de precio
</commit_message>
<xml_diff>
--- a/CursosIEDCH/public/CALCULADORA FISCAL FINAL modificado.xlsx
+++ b/CursosIEDCH/public/CALCULADORA FISCAL FINAL modificado.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\A. UMB JUAN MANUEL PLATAFORMAS DIGITALES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sergi\.gemini\antigravity\scratch\CursosIEDCH\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C030BEA1-90FF-4C8C-B509-E9CA84F3DCAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C64FCD6A-FBB8-4CE4-B117-32B12EAC4566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculadora Fiscal Simplificada" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>SIMULADOR DE RETENCIONES Y PAGOS (SIN EXPLICACIONES)</t>
   </si>
@@ -99,9 +99,6 @@
   </si>
   <si>
     <t>Total recibido</t>
-  </si>
-  <si>
-    <t>PLATAFORMA P MORAL CON RFC</t>
   </si>
   <si>
     <t>PLATAFORMA P MORAL SIN RFC</t>
@@ -627,33 +624,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:F31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:E31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" customWidth="1"/>
-    <col min="4" max="4" width="27.44140625" customWidth="1"/>
-    <col min="5" max="5" width="19.6640625" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" ht="24.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="19.2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -661,7 +657,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="16.8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -669,32 +665,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="D10" s="16" t="s">
         <v>26</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>27</v>
       </c>
       <c r="E10" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="F10" s="16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>5</v>
       </c>
@@ -714,12 +707,8 @@
         <f>$B$6*$B$7</f>
         <v>20000</v>
       </c>
-      <c r="F11" s="9">
-        <f>$B$6*$B$7</f>
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>20</v>
       </c>
@@ -736,15 +725,11 @@
         <v>17241.37931034483</v>
       </c>
       <c r="E12" s="9">
-        <f t="shared" ref="E12:F12" si="2">E11/1.16</f>
+        <f t="shared" ref="E12" si="2">E11/1.16</f>
         <v>17241.37931034483</v>
       </c>
-      <c r="F12" s="9">
-        <f t="shared" si="2"/>
-        <v>17241.37931034483</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>10</v>
       </c>
@@ -761,15 +746,11 @@
         <v>2758.620689655173</v>
       </c>
       <c r="E13" s="11">
-        <f t="shared" ref="E13:F13" si="5">E12*0.16</f>
+        <f t="shared" ref="E13" si="5">E12*0.16</f>
         <v>2758.620689655173</v>
       </c>
-      <c r="F13" s="11">
-        <f t="shared" si="5"/>
-        <v>2758.620689655173</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>21</v>
       </c>
@@ -786,18 +767,14 @@
         <v>20000.000000000004</v>
       </c>
       <c r="E14" s="11">
-        <f t="shared" ref="E14:F14" si="8">E12+E13</f>
+        <f t="shared" ref="E14" si="8">E12+E13</f>
         <v>20000.000000000004</v>
       </c>
-      <c r="F14" s="11">
-        <f t="shared" si="8"/>
-        <v>20000.000000000004</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
     </row>
-    <row r="16" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>11</v>
       </c>
@@ -814,15 +791,11 @@
         <v>20000.000000000004</v>
       </c>
       <c r="E16" s="9">
-        <f t="shared" ref="E16:F16" si="11">E14</f>
+        <f t="shared" ref="E16" si="11">E14</f>
         <v>20000.000000000004</v>
       </c>
-      <c r="F16" s="9">
-        <f t="shared" si="11"/>
-        <v>20000.000000000004</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>6</v>
       </c>
@@ -831,7 +804,7 @@
         <v>720</v>
       </c>
       <c r="C17" s="11">
-        <f t="shared" ref="C17:F17" si="12">C11*0.036</f>
+        <f t="shared" ref="C17:E17" si="12">C11*0.036</f>
         <v>720</v>
       </c>
       <c r="D17" s="11">
@@ -842,12 +815,8 @@
         <f t="shared" si="12"/>
         <v>720</v>
       </c>
-      <c r="F17" s="11">
-        <f t="shared" si="12"/>
-        <v>720</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>7</v>
       </c>
@@ -867,12 +836,8 @@
         <f>$B$7*3</f>
         <v>60</v>
       </c>
-      <c r="F18" s="13">
-        <f>$B$7*3</f>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>8</v>
       </c>
@@ -892,20 +857,15 @@
         <f t="shared" ref="E19" si="15">E11-E17-E18</f>
         <v>19220</v>
       </c>
-      <c r="F19" s="9">
-        <f t="shared" ref="F19" si="16">F11-F17-F18</f>
-        <v>19220</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-    </row>
-    <row r="21" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>9</v>
       </c>
@@ -925,12 +885,8 @@
         <f>E19*0.6</f>
         <v>11532</v>
       </c>
-      <c r="F21" s="20">
-        <f>F19*0.6</f>
-        <v>11532</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>17</v>
       </c>
@@ -938,9 +894,8 @@
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-    </row>
-    <row r="23" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>18</v>
       </c>
@@ -949,73 +904,61 @@
         <v>9941.3793103448279</v>
       </c>
       <c r="C23" s="9">
-        <f t="shared" ref="C23:D23" si="17">C21/1.16</f>
+        <f t="shared" ref="C23:D23" si="16">C21/1.16</f>
         <v>9941.3793103448279</v>
       </c>
       <c r="D23" s="9">
-        <f t="shared" si="17"/>
+        <f t="shared" si="16"/>
         <v>9941.3793103448279</v>
       </c>
       <c r="E23" s="9">
-        <f t="shared" ref="E23:F23" si="18">E21/1.16</f>
+        <f t="shared" ref="E23" si="17">E21/1.16</f>
         <v>9941.3793103448279</v>
       </c>
-      <c r="F23" s="9">
-        <f t="shared" si="18"/>
-        <v>9941.3793103448279</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>19</v>
       </c>
       <c r="B24" s="18">
-        <f t="shared" ref="B24" si="19">B23*0.16</f>
+        <f t="shared" ref="B24" si="18">B23*0.16</f>
         <v>1590.6206896551726</v>
       </c>
       <c r="C24" s="9">
-        <f t="shared" ref="C24:D24" si="20">C23*0.16</f>
+        <f t="shared" ref="C24:D24" si="19">C23*0.16</f>
         <v>1590.6206896551726</v>
       </c>
       <c r="D24" s="9">
-        <f t="shared" si="20"/>
+        <f t="shared" si="19"/>
         <v>1590.6206896551726</v>
       </c>
       <c r="E24" s="9">
-        <f t="shared" ref="E24" si="21">E23*0.16</f>
+        <f t="shared" ref="E24" si="20">E23*0.16</f>
         <v>1590.6206896551726</v>
       </c>
-      <c r="F24" s="9">
-        <f t="shared" ref="F24" si="22">F23*0.16</f>
-        <v>1590.6206896551726</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="25" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B25" s="18">
-        <f t="shared" ref="B25" si="23">B23+B24</f>
+        <f t="shared" ref="B25" si="21">B23+B24</f>
         <v>11532</v>
       </c>
       <c r="C25" s="9">
-        <f t="shared" ref="C25:D25" si="24">C23+C24</f>
+        <f t="shared" ref="C25:D25" si="22">C23+C24</f>
         <v>11532</v>
       </c>
       <c r="D25" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="22"/>
         <v>11532</v>
       </c>
       <c r="E25" s="9">
-        <f t="shared" ref="E25" si="25">E23+E24</f>
+        <f t="shared" ref="E25" si="23">E23+E24</f>
         <v>11532</v>
       </c>
-      <c r="F25" s="9">
-        <f t="shared" ref="F25" si="26">F23+F24</f>
-        <v>11532</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>12</v>
       </c>
@@ -1032,15 +975,11 @@
         <v>2306.4</v>
       </c>
       <c r="E26" s="17">
-        <f>E25*0.025</f>
-        <v>288.3</v>
-      </c>
-      <c r="F26" s="17">
-        <f>F25*0.2</f>
+        <f>E25*0.2</f>
         <v>2306.4</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
         <v>13</v>
       </c>
@@ -1057,73 +996,60 @@
         <v>1590.6206896551726</v>
       </c>
       <c r="E27" s="17">
-        <f t="shared" ref="E27" si="27">(E23*0.16)*0.5</f>
-        <v>795.31034482758628</v>
-      </c>
-      <c r="F27" s="17">
-        <f>(F23*0.16)*1</f>
+        <f>(E23*0.16)*1</f>
         <v>1590.6206896551726</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
       <c r="B28" s="17"/>
       <c r="C28" s="11"/>
       <c r="D28" s="11"/>
       <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-    </row>
-    <row r="29" spans="1:6" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="29" spans="1:5" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B29" s="17">
-        <f t="shared" ref="B29" si="28">B26+B27</f>
+        <f t="shared" ref="B29" si="24">B26+B27</f>
         <v>2054.5848620689658</v>
       </c>
       <c r="C29" s="11">
-        <f t="shared" ref="C29:D29" si="29">C26+C27</f>
+        <f t="shared" ref="C29:D29" si="25">C26+C27</f>
         <v>1083.6103448275862</v>
       </c>
       <c r="D29" s="11">
-        <f t="shared" si="29"/>
+        <f t="shared" si="25"/>
         <v>3897.0206896551726</v>
       </c>
       <c r="E29" s="11">
-        <f t="shared" ref="E29" si="30">E26+E27</f>
-        <v>1083.6103448275862</v>
-      </c>
-      <c r="F29" s="11">
-        <f t="shared" ref="F29" si="31">F26+F27</f>
+        <f t="shared" ref="E29" si="26">E26+E27</f>
         <v>3897.0206896551726</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="21.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" ht="21.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
         <v>15</v>
       </c>
       <c r="B30" s="19">
-        <f t="shared" ref="B30" si="32">B25-B29</f>
+        <f t="shared" ref="B30" si="27">B25-B29</f>
         <v>9477.4151379310351</v>
       </c>
       <c r="C30" s="15">
-        <f t="shared" ref="C30:D30" si="33">C25-C29</f>
+        <f t="shared" ref="C30:D30" si="28">C25-C29</f>
         <v>10448.389655172414</v>
       </c>
       <c r="D30" s="15">
-        <f t="shared" si="33"/>
+        <f t="shared" si="28"/>
         <v>7634.9793103448274</v>
       </c>
       <c r="E30" s="15">
-        <f t="shared" ref="E30" si="34">E25-E29</f>
-        <v>10448.389655172414</v>
-      </c>
-      <c r="F30" s="15">
-        <f t="shared" ref="F30" si="35">F25-F29</f>
+        <f t="shared" ref="E30" si="29">E25-E29</f>
         <v>7634.9793103448274</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="31" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>